<commit_message>
Actualizacion automatica del mapa (2026-03-11 15:32:54)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R178"/>
+  <dimension ref="A1:R185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13363,22 +13363,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>900008676910</t>
+          <t>-748</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>1/23/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ALVEAR, MARCELO T. DE 2101</t>
+          <t>GUTENBERG 340</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -13393,10 +13393,14 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr"/>
+          <t>812440623</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>inclinado base podrida</t>
+        </is>
+      </c>
       <c r="I152" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -13409,31 +13413,31 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.39773</v>
+        <v>-58.471395</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.597163</v>
+        <v>-34.592451</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>PUE-?</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -13445,7 +13449,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>-748</t>
+          <t>-749</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -13455,12 +13459,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>GUTENBERG 340</t>
+          <t>Moreno 2965</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -13475,12 +13479,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>812440623</t>
+          <t>812440614</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>inclinado base podrida</t>
+          <t xml:space="preserve">base corroida </t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -13495,31 +13499,31 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L153" t="n">
         <v>1</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.471395</v>
+        <v>-58.407758</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.592451</v>
+        <v>-34.613793</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>PUE-?</t>
+          <t>CEN-I</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -13531,7 +13535,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>-749</t>
+          <t>-750</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -13541,12 +13545,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Moreno 2965</t>
+          <t>JURAMENTO 4979</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -13561,12 +13565,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>812440614</t>
+          <t>812440599</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t xml:space="preserve">base corroida </t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -13588,24 +13592,24 @@
         <v>1</v>
       </c>
       <c r="M154" t="n">
-        <v>-58.407758</v>
+        <v>-58.481188</v>
       </c>
       <c r="N154" t="n">
-        <v>-34.613793</v>
+        <v>-34.577198</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>CEN-I</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -13617,7 +13621,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>-750</t>
+          <t>-752</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -13627,12 +13631,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>JURAMENTO 4979</t>
+          <t>RIVADAVIA AV. 5691</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -13647,7 +13651,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>812440599</t>
+          <t>812440563</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -13674,24 +13678,24 @@
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>-58.481188</v>
+        <v>-58.445685</v>
       </c>
       <c r="N155" t="n">
-        <v>-34.577198</v>
+        <v>-34.622144</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
@@ -13703,7 +13707,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>-752</t>
+          <t>-754</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -13713,12 +13717,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>RIVADAVIA AV. 5691</t>
+          <t>PINO, VIRREY DEL 1503</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -13733,7 +13737,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>812440563</t>
+          <t>812440515</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -13760,24 +13764,24 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-58.445685</v>
+        <v>-58.442723</v>
       </c>
       <c r="N156" t="n">
-        <v>-34.622144</v>
+        <v>-34.56085</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>BLO-A</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13789,7 +13793,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>-754</t>
+          <t>-755</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -13799,12 +13803,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>PINO, VIRREY DEL 1503</t>
+          <t>CONDE 4296</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -13819,12 +13823,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>812440515</t>
+          <t>812440509</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -13846,10 +13850,10 @@
         <v>1</v>
       </c>
       <c r="M157" t="n">
-        <v>-58.442723</v>
+        <v>-58.481187</v>
       </c>
       <c r="N157" t="n">
-        <v>-34.56085</v>
+        <v>-34.548301</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -13863,7 +13867,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>BLO-A</t>
+          <t>COG-P</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -13875,7 +13879,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>-755</t>
+          <t>-760</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -13885,12 +13889,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>CONDE 4296</t>
+          <t>MAZA 1615</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -13905,12 +13909,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>812440509</t>
+          <t>812440354</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>base corroida e inclinada</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -13932,24 +13936,24 @@
         <v>1</v>
       </c>
       <c r="M158" t="n">
-        <v>-58.481187</v>
+        <v>-58.414586</v>
       </c>
       <c r="N158" t="n">
-        <v>-34.548301</v>
+        <v>-34.630095</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>COG-P</t>
+          <t>PPT-E</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -13961,7 +13965,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>-760</t>
+          <t>-761</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -13971,12 +13975,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>MAZA 1615</t>
+          <t>MOLDES 2901</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -13991,12 +13995,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>812440354</t>
+          <t>812440341</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>base corroida e inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -14018,24 +14022,24 @@
         <v>1</v>
       </c>
       <c r="M159" t="n">
-        <v>-58.414586</v>
+        <v>-58.465305</v>
       </c>
       <c r="N159" t="n">
-        <v>-34.630095</v>
+        <v>-34.556794</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>PPT-E</t>
+          <t>COG-K</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14047,22 +14051,22 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>-761</t>
+          <t>-765</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/2/2026</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>MOLDES 2901</t>
+          <t>AVALOS 180</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -14077,7 +14081,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>812440341</t>
+          <t>812503657</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -14104,14 +14108,14 @@
         <v>1</v>
       </c>
       <c r="M160" t="n">
-        <v>-58.465305</v>
+        <v>-58.465874</v>
       </c>
       <c r="N160" t="n">
-        <v>-34.556794</v>
+        <v>-34.594613</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P160" t="inlineStr">
@@ -14121,7 +14125,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>COG-K</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14133,7 +14137,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>-765</t>
+          <t>-768</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14143,12 +14147,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>AVALOS 180</t>
+          <t>CONCORDIA 3581</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -14163,12 +14167,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>812503657</t>
+          <t>812503649</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -14183,17 +14187,17 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L161" t="n">
         <v>1</v>
       </c>
       <c r="M161" t="n">
-        <v>-58.465874</v>
+        <v>-58.502724</v>
       </c>
       <c r="N161" t="n">
-        <v>-34.594613</v>
+        <v>-34.599311</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -14207,7 +14211,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14219,7 +14223,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>-768</t>
+          <t>-767</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14229,7 +14233,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>CONCORDIA 3581</t>
+          <t>CONCORDIA 3525</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -14249,7 +14253,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>812503649</t>
+          <t>812503647</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -14276,10 +14280,10 @@
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>-58.502724</v>
+        <v>-58.502389</v>
       </c>
       <c r="N162" t="n">
-        <v>-34.599311</v>
+        <v>-34.599679</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -14305,7 +14309,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>-767</t>
+          <t>-769</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -14315,12 +14319,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>CONCORDIA 3525</t>
+          <t>RIVERA, PEDRO I., DR. 2734</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -14335,12 +14339,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>812503647</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -14350,26 +14354,26 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L163" t="n">
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>-58.502389</v>
+        <v>-58.464354</v>
       </c>
       <c r="N163" t="n">
-        <v>-34.599679</v>
+        <v>-34.5587</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -14379,7 +14383,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>COG-K</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -14391,22 +14395,22 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>-769</t>
+          <t>-770</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>3/2/2026</t>
+          <t>3/5/2026</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>RIVERA, PEDRO I., DR. 2734</t>
+          <t>SAN JUAN AV. 1245</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -14426,7 +14430,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -14436,7 +14440,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -14448,24 +14452,24 @@
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>-58.464354</v>
+        <v>-58.383649</v>
       </c>
       <c r="N164" t="n">
-        <v>-34.5587</v>
+        <v>-34.622187</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>COG-K</t>
+          <t>CEN-A</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -14477,22 +14481,22 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>-770</t>
+          <t>-771</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>3/5/2026</t>
+          <t>2/18/2026</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 1245</t>
+          <t>SAN BLAS 4112</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -14510,11 +14514,7 @@
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
+      <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -14522,36 +14522,36 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L165" t="n">
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.383649</v>
+        <v>-58.494458</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.622187</v>
+        <v>-34.620078</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>CEN-A</t>
+          <t>DEV-J</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14563,22 +14563,22 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>-771</t>
+          <t>-772</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2/18/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>SAN BLAS 4112</t>
+          <t>LA PLATA AV. 2304</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -14596,7 +14596,11 @@
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Desplazar Columna</t>
+        </is>
+      </c>
       <c r="I166" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -14609,31 +14613,31 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L166" t="n">
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.494458</v>
+        <v>-58.423086</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.620078</v>
+        <v>-34.641356</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>DEV-J</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -14645,17 +14649,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>-773</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>LA PLATA AV. 2244</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -14680,12 +14684,12 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>desmonte</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -14702,10 +14706,10 @@
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.423086</v>
+        <v>-58.423288</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.641356</v>
+        <v>-34.640581</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -14731,7 +14735,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>-773</t>
+          <t>-774</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -14741,12 +14745,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2244</t>
+          <t>CASEROS AV. 4131</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -14766,12 +14770,12 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>desmonte</t>
+          <t>mover a 4111</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -14788,10 +14792,10 @@
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.423288</v>
+        <v>-58.422741</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.640581</v>
+        <v>-34.639999</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -14817,22 +14821,22 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>8452</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>LIVERPOOL 2975</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -14852,7 +14856,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Columna Picada</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -14874,24 +14878,24 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>-58.422741</v>
+        <v>-58.483044</v>
       </c>
       <c r="N169" t="n">
-        <v>-34.639999</v>
+        <v>-34.583393</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -14903,7 +14907,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>8452</t>
+          <t>8453</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -14913,7 +14917,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>LIVERPOOL 2975</t>
+          <t xml:space="preserve">LIVERPOOL 2903 </t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -14960,10 +14964,10 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.483044</v>
+        <v>-58.482265</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.583393</v>
+        <v>-34.582718</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -14989,7 +14993,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>8453</t>
+          <t>8454</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -14999,7 +15003,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVERPOOL 2903 </t>
+          <t>BAUNESS 1600</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -15046,10 +15050,10 @@
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>-58.482265</v>
+        <v>-58.481148</v>
       </c>
       <c r="N171" t="n">
-        <v>-34.582718</v>
+        <v>-34.583622</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -15063,7 +15067,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15075,7 +15079,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>8454</t>
+          <t>8455</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -15085,7 +15089,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>BAUNESS 1600</t>
+          <t>LIVERPOOL 2849</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -15132,10 +15136,10 @@
         <v>1</v>
       </c>
       <c r="M172" t="n">
-        <v>-58.481148</v>
+        <v>-58.481371</v>
       </c>
       <c r="N172" t="n">
-        <v>-34.583622</v>
+        <v>-34.582578</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -15149,7 +15153,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15161,7 +15165,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>8455</t>
+          <t>8456</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -15171,7 +15175,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>LIVERPOOL 2849</t>
+          <t>LONDRES 4142</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -15218,10 +15222,10 @@
         <v>1</v>
       </c>
       <c r="M173" t="n">
-        <v>-58.481371</v>
+        <v>-58.479712</v>
       </c>
       <c r="N173" t="n">
-        <v>-34.582578</v>
+        <v>-34.581443</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -15235,7 +15239,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -15247,7 +15251,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>8456</t>
+          <t>8458</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -15257,7 +15261,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>LONDRES 4142</t>
+          <t>GAMARRA y TREVERIS</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -15295,19 +15299,15 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K174" t="inlineStr"/>
       <c r="L174" t="n">
         <v>1</v>
       </c>
       <c r="M174" t="n">
-        <v>-58.479712</v>
+        <v>-58.477099</v>
       </c>
       <c r="N174" t="n">
-        <v>-34.581443</v>
+        <v>-34.582525</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>8458</t>
+          <t>8460</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -15343,7 +15343,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>GAMARRA y TREVERIS</t>
+          <t>VICTORICA, BENJAMIN, GENERAL, AV. 2968</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -15381,15 +15381,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L175" t="n">
         <v>1</v>
       </c>
       <c r="M175" t="n">
-        <v>-58.477099</v>
+        <v>-58.479692</v>
       </c>
       <c r="N175" t="n">
-        <v>-34.582525</v>
+        <v>-34.586552</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -15403,7 +15407,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -15415,7 +15419,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t xml:space="preserve">8460 </t>
+          <t>8461</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -15425,7 +15429,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>VICTORICA, BENJAMIN, GENERAL, AV. 2968</t>
+          <t>BARZANA 1676</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -15463,19 +15467,15 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K176" t="inlineStr"/>
       <c r="L176" t="n">
         <v>1</v>
       </c>
       <c r="M176" t="n">
-        <v>-58.479692</v>
+        <v>-58.484405</v>
       </c>
       <c r="N176" t="n">
-        <v>-34.586552</v>
+        <v>-34.583582</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -15489,7 +15489,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -15501,7 +15501,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">8461 </t>
+          <t>8463</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -15511,12 +15511,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>BARZANA 1676</t>
+          <t>LA PAMPA 5896</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -15549,15 +15549,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L177" t="n">
         <v>1</v>
       </c>
       <c r="M177" t="n">
-        <v>-58.484405</v>
+        <v>-58.487925</v>
       </c>
       <c r="N177" t="n">
-        <v>-34.583582</v>
+        <v>-34.584375</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -15571,7 +15575,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-K</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -15583,22 +15587,22 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">8463 </t>
+          <t xml:space="preserve">8470 </t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/11/2026</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>LA PAMPA 5896</t>
+          <t>AV. GRAL.BENJAMIN VICTORICA 282</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -15611,14 +15615,10 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Columna Picada</t>
+          <t>Cambiar columna</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -15639,28 +15639,598 @@
       <c r="L178" t="n">
         <v>1</v>
       </c>
-      <c r="M178" t="n">
-        <v>-58.487925</v>
-      </c>
-      <c r="N178" t="n">
-        <v>-34.584375</v>
-      </c>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
       <c r="O178" t="inlineStr">
         <is>
+          <t>No ubicado</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>No clasificado, consultar con mantenimiento</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>No ubicado</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8471 </t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>BUCARELLI 1253</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Cambiar columna</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>1</v>
+      </c>
+      <c r="M179" t="n">
+        <v>-58.47844</v>
+      </c>
+      <c r="N179" t="n">
+        <v>-34.586982</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
           <t>Paternal</t>
         </is>
       </c>
-      <c r="P178" t="inlineStr">
+      <c r="P179" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q178" t="inlineStr">
-        <is>
-          <t>ATH-K</t>
-        </is>
-      </c>
-      <c r="R178" t="inlineStr">
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>ATH-G</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8473 </t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>VIRREY AVILES 3883</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>1</v>
+      </c>
+      <c r="M180" t="n">
+        <v>-58.46429</v>
+      </c>
+      <c r="N180" t="n">
+        <v>-34.578287</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>ATH-H</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8474 </t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>ESTOMBA 1327</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>1</v>
+      </c>
+      <c r="M181" t="n">
+        <v>-58.464844</v>
+      </c>
+      <c r="N181" t="n">
+        <v>-34.578243</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>ATH-G</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8475 </t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>AV. DE LOS INCAS 3594</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Columna Inclinada </t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>1</v>
+      </c>
+      <c r="M182" t="n">
+        <v>-58.463971</v>
+      </c>
+      <c r="N182" t="n">
+        <v>-34.575577</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>ATH-H</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8476 </t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>GIRIBONE 2219</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>1</v>
+      </c>
+      <c r="M183" t="n">
+        <v>-58.472418</v>
+      </c>
+      <c r="N183" t="n">
+        <v>-34.57958</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>ATH-E</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8568 </t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>HOLMBERG 1053</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Columna Cementar</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L184" t="n">
+        <v>1</v>
+      </c>
+      <c r="M184" t="n">
+        <v>-58.468422</v>
+      </c>
+      <c r="N184" t="n">
+        <v>-34.582173</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>ATH-F</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8569 </t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>3/11/2026</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>GARCIA DEL RIO 4577</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L185" t="n">
+        <v>1</v>
+      </c>
+      <c r="M185" t="n">
+        <v>-58.489649</v>
+      </c>
+      <c r="N185" t="n">
+        <v>-34.556653</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-13 11:06:08)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R185"/>
+  <dimension ref="A1:R205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14481,22 +14481,22 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>-771</t>
+          <t>-773</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2/18/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>SAN BLAS 4112</t>
+          <t>LA PLATA AV. 2244</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -14514,10 +14514,14 @@
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>desmonte</t>
+        </is>
+      </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -14527,31 +14531,31 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L165" t="n">
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.494458</v>
+        <v>-58.423288</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.620078</v>
+        <v>-34.640581</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>DEV-J</t>
+          <t>PPT-L</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14563,7 +14567,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>-772</t>
+          <t>8452</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -14573,12 +14577,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2304</t>
+          <t>LIVERPOOL 2975</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -14598,7 +14602,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Desplazar Columna</t>
+          <t>Columna Picada</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -14620,24 +14624,24 @@
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.423086</v>
+        <v>-58.483044</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.641356</v>
+        <v>-34.583393</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -14649,22 +14653,22 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>-773</t>
+          <t>8453</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LA PLATA AV. 2244</t>
+          <t xml:space="preserve">LIVERPOOL 2903 </t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -14684,12 +14688,12 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>desmonte</t>
+          <t>Columna Picada</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -14706,24 +14710,24 @@
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.423288</v>
+        <v>-58.482265</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.640581</v>
+        <v>-34.582718</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -14735,22 +14739,22 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>-774</t>
+          <t>8454</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/10/2026</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>CASEROS AV. 4131</t>
+          <t>BAUNESS 1600</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -14770,7 +14774,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>mover a 4111</t>
+          <t>Columna Picada</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -14792,24 +14796,24 @@
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.422741</v>
+        <v>-58.481148</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.639999</v>
+        <v>-34.583622</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>PPT-L</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -14821,7 +14825,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>8452</t>
+          <t>8455</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -14831,7 +14835,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>LIVERPOOL 2975</t>
+          <t>LIVERPOOL 2849</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -14878,10 +14882,10 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>-58.483044</v>
+        <v>-58.481371</v>
       </c>
       <c r="N169" t="n">
-        <v>-34.583393</v>
+        <v>-34.582578</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -14907,7 +14911,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>8453</t>
+          <t>8456</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -14917,7 +14921,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIVERPOOL 2903 </t>
+          <t>LONDRES 4142</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -14964,10 +14968,10 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.482265</v>
+        <v>-58.479712</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.582718</v>
+        <v>-34.581443</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -14981,7 +14985,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -14993,7 +14997,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>8454</t>
+          <t>8458</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -15003,7 +15007,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>BAUNESS 1600</t>
+          <t>GAMARRA y TREVERIS</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -15041,19 +15045,15 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K171" t="inlineStr"/>
       <c r="L171" t="n">
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>-58.481148</v>
+        <v>-58.477099</v>
       </c>
       <c r="N171" t="n">
-        <v>-34.583622</v>
+        <v>-34.582525</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -15079,7 +15079,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>8455</t>
+          <t>8460</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -15089,7 +15089,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>LIVERPOOL 2849</t>
+          <t>VICTORICA, BENJAMIN, GENERAL, AV. 2968</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -15136,10 +15136,10 @@
         <v>1</v>
       </c>
       <c r="M172" t="n">
-        <v>-58.481371</v>
+        <v>-58.479692</v>
       </c>
       <c r="N172" t="n">
-        <v>-34.582578</v>
+        <v>-34.586552</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -15153,7 +15153,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15165,7 +15165,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>8456</t>
+          <t>8461</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -15175,7 +15175,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>LONDRES 4142</t>
+          <t>BARZANA 1676</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -15213,19 +15213,15 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K173" t="inlineStr"/>
       <c r="L173" t="n">
         <v>1</v>
       </c>
       <c r="M173" t="n">
-        <v>-58.479712</v>
+        <v>-58.484405</v>
       </c>
       <c r="N173" t="n">
-        <v>-34.581443</v>
+        <v>-34.583582</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -15251,7 +15247,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>8458</t>
+          <t>8463</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -15261,12 +15257,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>GAMARRA y TREVERIS</t>
+          <t>LA PAMPA 5896</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -15299,15 +15295,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L174" t="n">
         <v>1</v>
       </c>
       <c r="M174" t="n">
-        <v>-58.477099</v>
+        <v>-58.487925</v>
       </c>
       <c r="N174" t="n">
-        <v>-34.582525</v>
+        <v>-34.584375</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -15321,7 +15321,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-K</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -15333,17 +15333,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>8460</t>
+          <t xml:space="preserve">8470 </t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/11/2026</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>VICTORICA, BENJAMIN, GENERAL, AV. 2968</t>
+          <t>AV. GRAL.BENJAMIN VICTORICA 282</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -15361,14 +15361,10 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Columna Picada</t>
+          <t>Cambiar columna</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -15389,25 +15385,21 @@
       <c r="L175" t="n">
         <v>1</v>
       </c>
-      <c r="M175" t="n">
-        <v>-58.479692</v>
-      </c>
-      <c r="N175" t="n">
-        <v>-34.586552</v>
-      </c>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
       <c r="O175" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -15419,17 +15411,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>8461</t>
+          <t xml:space="preserve">8471 </t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/11/2026</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>BARZANA 1676</t>
+          <t>BUCARELLI 1253</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -15447,14 +15439,10 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Columna Picada</t>
+          <t>Cambiar columna</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -15467,15 +15455,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L176" t="n">
         <v>1</v>
       </c>
       <c r="M176" t="n">
-        <v>-58.484405</v>
+        <v>-58.47844</v>
       </c>
       <c r="N176" t="n">
-        <v>-34.583582</v>
+        <v>-34.586982</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -15489,7 +15481,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -15501,22 +15493,22 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>8463</t>
+          <t xml:space="preserve">8473 </t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>3/10/2026</t>
+          <t>3/11/2026</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>LA PAMPA 5896</t>
+          <t>VIRREY AVILES 3883</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -15529,19 +15521,15 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
+      <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Columna Picada</t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -15551,21 +15539,21 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L177" t="n">
         <v>1</v>
       </c>
       <c r="M177" t="n">
-        <v>-58.487925</v>
+        <v>-58.46429</v>
       </c>
       <c r="N177" t="n">
-        <v>-34.584375</v>
+        <v>-34.578287</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P177" t="inlineStr">
@@ -15575,7 +15563,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>ATH-K</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -15587,7 +15575,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">8470 </t>
+          <t xml:space="preserve">8474 </t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -15597,7 +15585,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>AV. GRAL.BENJAMIN VICTORICA 282</t>
+          <t>ESTOMBA 1327</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -15618,42 +15606,46 @@
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Cambiar columna</t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L178" t="n">
         <v>1</v>
       </c>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
+      <c r="M178" t="n">
+        <v>-58.464844</v>
+      </c>
+      <c r="N178" t="n">
+        <v>-34.578243</v>
+      </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -15665,7 +15657,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">8471 </t>
+          <t xml:space="preserve">8475 </t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -15675,7 +15667,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>BUCARELLI 1253</t>
+          <t>AV. DE LOS INCAS 3594</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -15696,12 +15688,12 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Cambiar columna</t>
+          <t xml:space="preserve">Columna Inclinada </t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -15718,14 +15710,14 @@
         <v>1</v>
       </c>
       <c r="M179" t="n">
-        <v>-58.47844</v>
+        <v>-58.463971</v>
       </c>
       <c r="N179" t="n">
-        <v>-34.586982</v>
+        <v>-34.575577</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P179" t="inlineStr">
@@ -15735,7 +15727,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -15747,7 +15739,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">8473 </t>
+          <t xml:space="preserve">8476 </t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -15757,7 +15749,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>VIRREY AVILES 3883</t>
+          <t>GIRIBONE 2219</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -15793,17 +15785,17 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L180" t="n">
         <v>1</v>
       </c>
       <c r="M180" t="n">
-        <v>-58.46429</v>
+        <v>-58.472418</v>
       </c>
       <c r="N180" t="n">
-        <v>-34.578287</v>
+        <v>-34.57958</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -15817,7 +15809,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>ATH-E</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -15829,7 +15821,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">8474 </t>
+          <t xml:space="preserve">8568 </t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -15839,12 +15831,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ESTOMBA 1327</t>
+          <t>HOLMBERG 1053</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -15860,7 +15852,7 @@
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Columna Inclinada</t>
+          <t>Columna Cementar</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -15870,22 +15862,22 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L181" t="n">
         <v>1</v>
       </c>
       <c r="M181" t="n">
-        <v>-58.464844</v>
+        <v>-58.468422</v>
       </c>
       <c r="N181" t="n">
-        <v>-34.578243</v>
+        <v>-34.582173</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -15899,7 +15891,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -15911,7 +15903,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">8475 </t>
+          <t xml:space="preserve">8569 </t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -15921,12 +15913,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>AV. DE LOS INCAS 3594</t>
+          <t>GARCIA DEL RIO 4577</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -15942,7 +15934,7 @@
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Columna Inclinada </t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -15964,14 +15956,14 @@
         <v>1</v>
       </c>
       <c r="M182" t="n">
-        <v>-58.463971</v>
+        <v>-58.489649</v>
       </c>
       <c r="N182" t="n">
-        <v>-34.575577</v>
+        <v>-34.556653</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P182" t="inlineStr">
@@ -15981,7 +15973,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>COG-O</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -15993,22 +15985,22 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">8476 </t>
+          <t xml:space="preserve">8574 </t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>3/11/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>GIRIBONE 2219</t>
+          <t xml:space="preserve">MANZANARES 4746 </t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -16046,14 +16038,14 @@
         <v>1</v>
       </c>
       <c r="M183" t="n">
-        <v>-58.472418</v>
+        <v>-58.490797</v>
       </c>
       <c r="N183" t="n">
-        <v>-34.57958</v>
+        <v>-34.558302</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P183" t="inlineStr">
@@ -16063,7 +16055,7 @@
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>ATH-E</t>
+          <t>COG-O</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -16075,17 +16067,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">8568 </t>
+          <t xml:space="preserve">8575 </t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>3/11/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>HOLMBERG 1053</t>
+          <t>LUGONES 3806</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -16106,7 +16098,7 @@
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Columna Cementar</t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -16128,14 +16120,14 @@
         <v>1</v>
       </c>
       <c r="M184" t="n">
-        <v>-58.468422</v>
+        <v>-58.490494</v>
       </c>
       <c r="N184" t="n">
-        <v>-34.582173</v>
+        <v>-34.557966</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P184" t="inlineStr">
@@ -16145,7 +16137,7 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>COG-O</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
@@ -16157,17 +16149,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">8569 </t>
+          <t>8576</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>3/11/2026</t>
+          <t>3/13/2026</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>GARCIA DEL RIO 4577</t>
+          <t>LUGONES 3866</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -16210,10 +16202,10 @@
         <v>1</v>
       </c>
       <c r="M185" t="n">
-        <v>-58.489649</v>
+        <v>-58.490728</v>
       </c>
       <c r="N185" t="n">
-        <v>-34.556653</v>
+        <v>-34.55763</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -16227,10 +16219,1650 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>8577</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUGONES 3992 </t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L186" t="n">
+        <v>1</v>
+      </c>
+      <c r="M186" t="n">
+        <v>-58.491397</v>
+      </c>
+      <c r="N186" t="n">
+        <v>-34.556668</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>8578</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUGONES 4030 </t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L187" t="n">
+        <v>1</v>
+      </c>
+      <c r="M187" t="n">
+        <v>-58.491655</v>
+      </c>
+      <c r="N187" t="n">
+        <v>-34.556298</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>8579</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>LUGONES 4090</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L188" t="n">
+        <v>1</v>
+      </c>
+      <c r="M188" t="n">
+        <v>-58.49191</v>
+      </c>
+      <c r="N188" t="n">
+        <v>-34.555928</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>8580</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>PAROISSIEN 4711</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L189" t="n">
+        <v>1</v>
+      </c>
+      <c r="M189" t="n">
+        <v>-58.491698</v>
+      </c>
+      <c r="N189" t="n">
+        <v>-34.556615</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>8581</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>MILLER 4016</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L190" t="n">
+        <v>1</v>
+      </c>
+      <c r="M190" t="n">
+        <v>-58.492605</v>
+      </c>
+      <c r="N190" t="n">
+        <v>-34.556761</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>8583</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>ACHA MARIANO GRAL 3712</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Sin chequear</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L191" t="n">
+        <v>1</v>
+      </c>
+      <c r="M191" t="n">
+        <v>-58.489045</v>
+      </c>
+      <c r="N191" t="n">
+        <v>-34.558226</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
           <t>COG-O</t>
         </is>
       </c>
-      <c r="R185" t="inlineStr">
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>8584</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>ACHA MARIANO GRAL 3744</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>1</v>
+      </c>
+      <c r="M192" t="n">
+        <v>-58.489142</v>
+      </c>
+      <c r="N192" t="n">
+        <v>-34.558086</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>8585</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>MANZANARES 4512</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L193" t="n">
+        <v>1</v>
+      </c>
+      <c r="M193" t="n">
+        <v>-58.488739</v>
+      </c>
+      <c r="N193" t="n">
+        <v>-34.557321</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>8586</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>MACHAIN 3709</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L194" t="n">
+        <v>1</v>
+      </c>
+      <c r="M194" t="n">
+        <v>-58.488038</v>
+      </c>
+      <c r="N194" t="n">
+        <v>-34.557763</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>8587</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>ACHA MARIANO GRAL 3802</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L195" t="n">
+        <v>1</v>
+      </c>
+      <c r="M195" t="n">
+        <v>-58.489543</v>
+      </c>
+      <c r="N195" t="n">
+        <v>-34.557511</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>COG-O</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>8588</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>ACHA MARIANO GRAL 3874</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L196" t="n">
+        <v>1</v>
+      </c>
+      <c r="M196" t="n">
+        <v>-58.489778</v>
+      </c>
+      <c r="N196" t="n">
+        <v>-34.557174</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>8589</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>ACHA MARIANO GRAL 3948</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L197" t="n">
+        <v>1</v>
+      </c>
+      <c r="M197" t="n">
+        <v>-58.490224</v>
+      </c>
+      <c r="N197" t="n">
+        <v>-34.556533</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>COG-A</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>8597</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>JUJUY AV 1717</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L198" t="n">
+        <v>1</v>
+      </c>
+      <c r="M198" t="n">
+        <v>-58.400922</v>
+      </c>
+      <c r="N198" t="n">
+        <v>-34.630312</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>PPT-F</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>8598</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>IGUAZU 590</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L199" t="n">
+        <v>1</v>
+      </c>
+      <c r="M199" t="n">
+        <v>-58.405605</v>
+      </c>
+      <c r="N199" t="n">
+        <v>-34.644231</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>PPT-K</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>8602</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIAZ CNEL AV 2139 </t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L200" t="n">
+        <v>1</v>
+      </c>
+      <c r="M200" t="n">
+        <v>-58.408769</v>
+      </c>
+      <c r="N200" t="n">
+        <v>-34.587342</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>AGU-J</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>8605</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>CONDE 3080</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L201" t="n">
+        <v>1</v>
+      </c>
+      <c r="M201" t="n">
+        <v>-58.47322</v>
+      </c>
+      <c r="N201" t="n">
+        <v>-34.558645</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>COG-L</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>8606</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>YRIGOYEN HIPOLITO 1934</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L202" t="n">
+        <v>1</v>
+      </c>
+      <c r="M202" t="n">
+        <v>-58.394029</v>
+      </c>
+      <c r="N202" t="n">
+        <v>-34.610507</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>CEN-G</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>8609</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>SEGUI JUAN FRANCISCO 4691</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L203" t="n">
+        <v>1</v>
+      </c>
+      <c r="M203" t="n">
+        <v>-58.422229</v>
+      </c>
+      <c r="N203" t="n">
+        <v>-34.573148</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>VCR-M</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>8610</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>GANDHI MAHATMA 295</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Columna Inclinada</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L204" t="n">
+        <v>1</v>
+      </c>
+      <c r="M204" t="n">
+        <v>-58.440568</v>
+      </c>
+      <c r="N204" t="n">
+        <v>-34.6034</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>ALM-N</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>8615</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>3/13/2026</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>AGUIRRE 794</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L205" t="n">
+        <v>1</v>
+      </c>
+      <c r="M205" t="n">
+        <v>-58.438085</v>
+      </c>
+      <c r="N205" t="n">
+        <v>-34.595145</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>VCR-H</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-18 10:10:50)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R205"/>
+  <dimension ref="A1:R207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17215,7 +17215,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>8597</t>
+          <t>8598</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>JUJUY AV 1717</t>
+          <t>IGUAZU 590</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -17268,10 +17268,10 @@
         <v>1</v>
       </c>
       <c r="M198" t="n">
-        <v>-58.400922</v>
+        <v>-58.405605</v>
       </c>
       <c r="N198" t="n">
-        <v>-34.630312</v>
+        <v>-34.644231</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -17285,7 +17285,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>PPT-F</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -17297,7 +17297,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>8598</t>
+          <t>8602</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -17307,12 +17307,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>IGUAZU 590</t>
+          <t xml:space="preserve">DIAZ CNEL AV 2139 </t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -17350,14 +17350,14 @@
         <v>1</v>
       </c>
       <c r="M199" t="n">
-        <v>-58.405605</v>
+        <v>-58.408769</v>
       </c>
       <c r="N199" t="n">
-        <v>-34.644231</v>
+        <v>-34.587342</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P199" t="inlineStr">
@@ -17367,7 +17367,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>PPT-K</t>
+          <t>AGU-J</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -17379,7 +17379,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>8602</t>
+          <t>8605</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -17389,12 +17389,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIAZ CNEL AV 2139 </t>
+          <t>CONDE 3080</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -17432,24 +17432,24 @@
         <v>1</v>
       </c>
       <c r="M200" t="n">
-        <v>-58.408769</v>
+        <v>-58.47322</v>
       </c>
       <c r="N200" t="n">
-        <v>-34.587342</v>
+        <v>-34.558645</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>AGU-J</t>
+          <t>COG-L</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -17461,7 +17461,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>8605</t>
+          <t>8606</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -17471,12 +17471,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>CONDE 3080</t>
+          <t>YRIGOYEN HIPOLITO 1934</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -17514,24 +17514,24 @@
         <v>1</v>
       </c>
       <c r="M201" t="n">
-        <v>-58.47322</v>
+        <v>-58.394029</v>
       </c>
       <c r="N201" t="n">
-        <v>-34.558645</v>
+        <v>-34.610507</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>COG-L</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">
@@ -17543,7 +17543,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>8606</t>
+          <t>8609</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -17553,12 +17553,12 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>YRIGOYEN HIPOLITO 1934</t>
+          <t>SEGUI JUAN FRANCISCO 4691</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -17596,14 +17596,14 @@
         <v>1</v>
       </c>
       <c r="M202" t="n">
-        <v>-58.394029</v>
+        <v>-58.422229</v>
       </c>
       <c r="N202" t="n">
-        <v>-34.610507</v>
+        <v>-34.573148</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P202" t="inlineStr">
@@ -17613,7 +17613,7 @@
       </c>
       <c r="Q202" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>VCR-M</t>
         </is>
       </c>
       <c r="R202" t="inlineStr">
@@ -17625,7 +17625,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>8609</t>
+          <t>8610</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -17635,12 +17635,12 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>SEGUI JUAN FRANCISCO 4691</t>
+          <t>GANDHI MAHATMA 295</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -17656,12 +17656,12 @@
       <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>Columna Inclinada</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -17678,24 +17678,24 @@
         <v>1</v>
       </c>
       <c r="M203" t="n">
-        <v>-58.422229</v>
+        <v>-58.440568</v>
       </c>
       <c r="N203" t="n">
-        <v>-34.573148</v>
+        <v>-34.6034</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q203" t="inlineStr">
         <is>
-          <t>VCR-M</t>
+          <t>ALM-N</t>
         </is>
       </c>
       <c r="R203" t="inlineStr">
@@ -17707,7 +17707,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>8610</t>
+          <t>8615</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -17717,7 +17717,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>GANDHI MAHATMA 295</t>
+          <t>AGUIRRE 794</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -17738,12 +17738,12 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Columna Inclinada</t>
+          <t>Cambiar Columna</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -17760,24 +17760,24 @@
         <v>1</v>
       </c>
       <c r="M204" t="n">
-        <v>-58.440568</v>
+        <v>-58.438085</v>
       </c>
       <c r="N204" t="n">
-        <v>-34.6034</v>
+        <v>-34.595145</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q204" t="inlineStr">
         <is>
-          <t>ALM-N</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R204" t="inlineStr">
@@ -17789,22 +17789,22 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>8615</t>
+          <t xml:space="preserve">8618 </t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>3/13/2026</t>
+          <t>3/17/2026</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>AGUIRRE 794</t>
+          <t>VALLEJOS 4319</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -17820,7 +17820,7 @@
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
-          <t>Cambiar Columna</t>
+          <t>Cambiar Poste de madera a PRFV</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -17833,36 +17833,196 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K205" t="inlineStr"/>
       <c r="L205" t="n">
         <v>1</v>
       </c>
       <c r="M205" t="n">
-        <v>-58.438085</v>
+        <v>-58.51875</v>
       </c>
       <c r="N205" t="n">
-        <v>-34.595145</v>
+        <v>-34.598858</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P205" t="inlineStr">
         <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>PUE-P</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8619 </t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>3/17/2026</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>CONCORDIA 3575</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Desmontar Poste y migrar a Columna</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Desmonte</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L206" t="n">
+        <v>1</v>
+      </c>
+      <c r="M206" t="n">
+        <v>-58.502664</v>
+      </c>
+      <c r="N206" t="n">
+        <v>-34.599377</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>PUE-B</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8623    </t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>3/17/2026</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>INCLAN 2402</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr"/>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Cambiar Columna</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L207" t="n">
+        <v>1</v>
+      </c>
+      <c r="M207" t="n">
+        <v>-58.398304</v>
+      </c>
+      <c r="N207" t="n">
+        <v>-34.629576</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q205" t="inlineStr">
-        <is>
-          <t>VCR-H</t>
-        </is>
-      </c>
-      <c r="R205" t="inlineStr">
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>PPT-F</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-23 13:58:30)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R237"/>
+  <dimension ref="A1:R243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20069,7 +20069,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>8684</t>
+          <t>00223023</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -20079,12 +20079,12 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 727</t>
+          <t>SAN JUAN AV. 2201</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -20097,7 +20097,11 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G233" t="inlineStr"/>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
       <c r="H233" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -20122,14 +20126,14 @@
         <v>1</v>
       </c>
       <c r="M233" t="n">
-        <v>-58.425539</v>
+        <v>-58.396491</v>
       </c>
       <c r="N233" t="n">
-        <v>-34.602286</v>
+        <v>-34.622986</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P233" t="inlineStr">
@@ -20139,7 +20143,7 @@
       </c>
       <c r="Q233" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>CEN-B</t>
         </is>
       </c>
       <c r="R233" t="inlineStr">
@@ -20151,7 +20155,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>00223023</t>
+          <t>00275970</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -20161,7 +20165,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 2201</t>
+          <t xml:space="preserve"> JUJUY AV. 252</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -20179,11 +20183,7 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G234" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
+      <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -20208,14 +20208,14 @@
         <v>1</v>
       </c>
       <c r="M234" t="n">
-        <v>-58.396491</v>
+        <v>-58.405319</v>
       </c>
       <c r="N234" t="n">
-        <v>-34.622986</v>
+        <v>-34.612931</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P234" t="inlineStr">
@@ -20225,7 +20225,7 @@
       </c>
       <c r="Q234" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>CEN-H</t>
         </is>
       </c>
       <c r="R234" t="inlineStr">
@@ -20237,7 +20237,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>00275970</t>
+          <t>00283507</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -20247,12 +20247,12 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JUJUY AV. 252</t>
+          <t xml:space="preserve">HERRERA 475 </t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -20290,14 +20290,14 @@
         <v>1</v>
       </c>
       <c r="M235" t="n">
-        <v>-58.405319</v>
+        <v>-58.378709</v>
       </c>
       <c r="N235" t="n">
-        <v>-34.612931</v>
+        <v>-34.635064</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P235" t="inlineStr">
@@ -20307,7 +20307,7 @@
       </c>
       <c r="Q235" t="inlineStr">
         <is>
-          <t>CEN-H</t>
+          <t>CON-H</t>
         </is>
       </c>
       <c r="R235" t="inlineStr">
@@ -20319,7 +20319,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>00283507</t>
+          <t>00289536</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -20329,12 +20329,12 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERRERA 475 </t>
+          <t>VALDENEGRO 3554</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -20372,24 +20372,24 @@
         <v>1</v>
       </c>
       <c r="M236" t="n">
-        <v>-58.378709</v>
+        <v>-58.490576</v>
       </c>
       <c r="N236" t="n">
-        <v>-34.635064</v>
+        <v>-34.561508</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q236" t="inlineStr">
         <is>
-          <t>CON-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R236" t="inlineStr">
@@ -20401,22 +20401,22 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>00289536</t>
+          <t>00317296</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/23/2026</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>VALDENEGRO 3554</t>
+          <t>AGRELO 3620</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -20454,27 +20454,519 @@
         <v>1</v>
       </c>
       <c r="M237" t="n">
-        <v>-58.490576</v>
+        <v>-58.417002</v>
       </c>
       <c r="N237" t="n">
-        <v>-34.561508</v>
+        <v>-34.618613</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>ALM-B</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>00322642</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>3/23/2026</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>ESTADO DE PALESTINA 727</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L238" t="n">
+        <v>1</v>
+      </c>
+      <c r="M238" t="n">
+        <v>-58.425539</v>
+      </c>
+      <c r="N238" t="n">
+        <v>-34.602286</v>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>CLI-N</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>8263</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>3/23/2026</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>MEXICO 3306</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr"/>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L239" t="n">
+        <v>1</v>
+      </c>
+      <c r="M239" t="n">
+        <v>-58.412865</v>
+      </c>
+      <c r="N239" t="n">
+        <v>-34.619484</v>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>CEN-J</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>8265</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>3/23/2026</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>HUMBERTO 1 1999</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr"/>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L240" t="n">
+        <v>1</v>
+      </c>
+      <c r="M240" t="n">
+        <v>-58.394304</v>
+      </c>
+      <c r="N240" t="n">
+        <v>-34.621645</v>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>CEN-B</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>08672</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>3/23/2026</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>HERRERA 540</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr"/>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L241" t="n">
+        <v>1</v>
+      </c>
+      <c r="M241" t="n">
+        <v>-58.378264</v>
+      </c>
+      <c r="N241" t="n">
+        <v>-34.636021</v>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>CON-H</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>8647</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>3/24/2026</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MELIAN AV 4827 </t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr"/>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L242" t="n">
+        <v>1</v>
+      </c>
+      <c r="M242" t="n">
+        <v>-58.487048</v>
+      </c>
+      <c r="N242" t="n">
+        <v>-34.545509</v>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
           <t>Saavedra</t>
         </is>
       </c>
-      <c r="P237" t="inlineStr">
+      <c r="P242" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q237" t="inlineStr">
-        <is>
-          <t>PUE-F</t>
-        </is>
-      </c>
-      <c r="R237" t="inlineStr">
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>COG-Q</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>8674</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>3/23/2026</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>BRASIL 2509</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L243" t="n">
+        <v>1</v>
+      </c>
+      <c r="M243" t="n">
+        <v>-58.399415</v>
+      </c>
+      <c r="N243" t="n">
+        <v>-34.631112</v>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>PPT-F</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-27 12:53:34)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R243"/>
+  <dimension ref="A1:R242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19003,7 +19003,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>00201041</t>
+          <t>8658</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -19013,12 +19013,12 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>HABANA 4448</t>
+          <t>REPUBLICA BOLIVARIANA DE VENEZUELA 2071</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -19034,7 +19034,7 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
-          <t>DEMONTAR POSTE Y REEMPLAZAR POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -19056,24 +19056,24 @@
         <v>1</v>
       </c>
       <c r="M220" t="n">
-        <v>-58.518808</v>
+        <v>-58.395567</v>
       </c>
       <c r="N220" t="n">
-        <v>-34.601236</v>
+        <v>-34.615169</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q220" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>CEN-C</t>
         </is>
       </c>
       <c r="R220" t="inlineStr">
@@ -19085,7 +19085,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>8658</t>
+          <t>8663</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -19095,12 +19095,12 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>REPUBLICA BOLIVARIANA DE VENEZUELA 2071</t>
+          <t>MONTENEGRO 1539</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -19116,12 +19116,12 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -19138,24 +19138,24 @@
         <v>1</v>
       </c>
       <c r="M221" t="n">
-        <v>-58.395567</v>
+        <v>-58.468478</v>
       </c>
       <c r="N221" t="n">
-        <v>-34.615169</v>
+        <v>-34.587599</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P221" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q221" t="inlineStr">
         <is>
-          <t>CEN-C</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R221" t="inlineStr">
@@ -19167,7 +19167,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>8663</t>
+          <t>8664</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -19177,7 +19177,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>MONTENEGRO 1539</t>
+          <t>JEREZ PEDRO DE 430</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -19220,10 +19220,10 @@
         <v>1</v>
       </c>
       <c r="M222" t="n">
-        <v>-58.468478</v>
+        <v>-58.467418</v>
       </c>
       <c r="N222" t="n">
-        <v>-34.587599</v>
+        <v>-34.586278</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -19249,7 +19249,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>8664</t>
+          <t>8668</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -19259,12 +19259,12 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>JEREZ PEDRO DE 430</t>
+          <t>GARCIA DEL RIO 4457</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -19302,14 +19302,14 @@
         <v>1</v>
       </c>
       <c r="M223" t="n">
-        <v>-58.467418</v>
+        <v>-58.488608</v>
       </c>
       <c r="N223" t="n">
-        <v>-34.586278</v>
+        <v>-34.556155</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P223" t="inlineStr">
@@ -19319,7 +19319,7 @@
       </c>
       <c r="Q223" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>COG-O</t>
         </is>
       </c>
       <c r="R223" t="inlineStr">
@@ -19331,7 +19331,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>8668</t>
+          <t>8667</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -19341,7 +19341,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>GARCIA DEL RIO 4457</t>
+          <t>MACHAIN 3817</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -19384,10 +19384,10 @@
         <v>1</v>
       </c>
       <c r="M224" t="n">
-        <v>-58.488608</v>
+        <v>-58.488586</v>
       </c>
       <c r="N224" t="n">
-        <v>-34.556155</v>
+        <v>-34.556965</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -19413,7 +19413,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>8667</t>
+          <t>8669</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -19423,7 +19423,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>MACHAIN 3817</t>
+          <t>MACHAIN 3961</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -19466,10 +19466,10 @@
         <v>1</v>
       </c>
       <c r="M225" t="n">
-        <v>-58.488586</v>
+        <v>-58.489299</v>
       </c>
       <c r="N225" t="n">
-        <v>-34.556965</v>
+        <v>-34.555926</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -19483,7 +19483,7 @@
       </c>
       <c r="Q225" t="inlineStr">
         <is>
-          <t>COG-O</t>
+          <t>COG-A</t>
         </is>
       </c>
       <c r="R225" t="inlineStr">
@@ -19495,7 +19495,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>8669</t>
+          <t>8671</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -19505,7 +19505,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>MACHAIN 3961</t>
+          <t>TRONADOR 284</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -19548,14 +19548,14 @@
         <v>1</v>
       </c>
       <c r="M226" t="n">
-        <v>-58.489299</v>
+        <v>-58.470504</v>
       </c>
       <c r="N226" t="n">
-        <v>-34.555926</v>
+        <v>-34.588131</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P226" t="inlineStr">
@@ -19565,7 +19565,7 @@
       </c>
       <c r="Q226" t="inlineStr">
         <is>
-          <t>COG-A</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R226" t="inlineStr">
@@ -19577,7 +19577,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>8671</t>
+          <t>8673</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -19587,12 +19587,12 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>TRONADOR 284</t>
+          <t>CADIZ 3715</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -19630,10 +19630,10 @@
         <v>1</v>
       </c>
       <c r="M227" t="n">
-        <v>-58.470504</v>
+        <v>-58.474682</v>
       </c>
       <c r="N227" t="n">
-        <v>-34.588131</v>
+        <v>-34.581396</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -19647,7 +19647,7 @@
       </c>
       <c r="Q227" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R227" t="inlineStr">
@@ -19659,7 +19659,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>8673</t>
+          <t>8675</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -19669,7 +19669,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>CADIZ 3715</t>
+          <t>LA HAYA 3722</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -19712,10 +19712,10 @@
         <v>1</v>
       </c>
       <c r="M228" t="n">
-        <v>-58.474682</v>
+        <v>-58.475097</v>
       </c>
       <c r="N228" t="n">
-        <v>-34.581396</v>
+        <v>-34.581101</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -19741,7 +19741,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>8675</t>
+          <t>8676</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -19751,12 +19751,12 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>LA HAYA 3722</t>
+          <t>HOLMBERG 979</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -19794,14 +19794,14 @@
         <v>1</v>
       </c>
       <c r="M229" t="n">
-        <v>-58.475097</v>
+        <v>-58.468449</v>
       </c>
       <c r="N229" t="n">
-        <v>-34.581101</v>
+        <v>-34.582898</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P229" t="inlineStr">
@@ -19811,7 +19811,7 @@
       </c>
       <c r="Q229" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R229" t="inlineStr">
@@ -19823,7 +19823,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>8676</t>
+          <t>8681</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -19833,12 +19833,12 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>HOLMBERG 979</t>
+          <t>GIRARDOT 1384</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -19854,12 +19854,12 @@
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
@@ -19876,10 +19876,10 @@
         <v>1</v>
       </c>
       <c r="M230" t="n">
-        <v>-58.468449</v>
+        <v>-58.466063</v>
       </c>
       <c r="N230" t="n">
-        <v>-34.582898</v>
+        <v>-34.587896</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -19905,7 +19905,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>8681</t>
+          <t>8682</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -19915,12 +19915,12 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>GIRARDOT 1384</t>
+          <t>CORRIENTES AV 4073</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -19958,24 +19958,24 @@
         <v>1</v>
       </c>
       <c r="M231" t="n">
-        <v>-58.466063</v>
+        <v>-58.422076</v>
       </c>
       <c r="N231" t="n">
-        <v>-34.587896</v>
+        <v>-34.60298</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P231" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q231" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>CLI-K</t>
         </is>
       </c>
       <c r="R231" t="inlineStr">
@@ -19987,7 +19987,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>8682</t>
+          <t>00223023</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -19997,12 +19997,12 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>CORRIENTES AV 4073</t>
+          <t>SAN JUAN AV. 2201</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -20015,7 +20015,11 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G232" t="inlineStr"/>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
       <c r="H232" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -20040,14 +20044,14 @@
         <v>1</v>
       </c>
       <c r="M232" t="n">
-        <v>-58.422076</v>
+        <v>-58.396491</v>
       </c>
       <c r="N232" t="n">
-        <v>-34.60298</v>
+        <v>-34.622986</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P232" t="inlineStr">
@@ -20057,7 +20061,7 @@
       </c>
       <c r="Q232" t="inlineStr">
         <is>
-          <t>CLI-K</t>
+          <t>CEN-B</t>
         </is>
       </c>
       <c r="R232" t="inlineStr">
@@ -20069,7 +20073,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>00223023</t>
+          <t>00275970</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -20079,7 +20083,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>SAN JUAN AV. 2201</t>
+          <t xml:space="preserve"> JUJUY AV. 252</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -20097,11 +20101,7 @@
           <t>Sin Asignar</t>
         </is>
       </c>
-      <c r="G233" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
+      <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -20126,14 +20126,14 @@
         <v>1</v>
       </c>
       <c r="M233" t="n">
-        <v>-58.396491</v>
+        <v>-58.405319</v>
       </c>
       <c r="N233" t="n">
-        <v>-34.622986</v>
+        <v>-34.612931</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P233" t="inlineStr">
@@ -20143,7 +20143,7 @@
       </c>
       <c r="Q233" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>CEN-H</t>
         </is>
       </c>
       <c r="R233" t="inlineStr">
@@ -20155,7 +20155,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>00275970</t>
+          <t>00283507</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -20165,12 +20165,12 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JUJUY AV. 252</t>
+          <t xml:space="preserve">HERRERA 475 </t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -20208,14 +20208,14 @@
         <v>1</v>
       </c>
       <c r="M234" t="n">
-        <v>-58.405319</v>
+        <v>-58.378709</v>
       </c>
       <c r="N234" t="n">
-        <v>-34.612931</v>
+        <v>-34.635064</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P234" t="inlineStr">
@@ -20225,7 +20225,7 @@
       </c>
       <c r="Q234" t="inlineStr">
         <is>
-          <t>CEN-H</t>
+          <t>CON-H</t>
         </is>
       </c>
       <c r="R234" t="inlineStr">
@@ -20237,7 +20237,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>00283507</t>
+          <t>00289536</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -20247,12 +20247,12 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t xml:space="preserve">HERRERA 475 </t>
+          <t>VALDENEGRO 3554</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -20290,24 +20290,24 @@
         <v>1</v>
       </c>
       <c r="M235" t="n">
-        <v>-58.378709</v>
+        <v>-58.490576</v>
       </c>
       <c r="N235" t="n">
-        <v>-34.635064</v>
+        <v>-34.561508</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q235" t="inlineStr">
         <is>
-          <t>CON-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R235" t="inlineStr">
@@ -20319,22 +20319,22 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>00289536</t>
+          <t>00317296</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>3/23/2026</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>VALDENEGRO 3554</t>
+          <t>AGRELO 3620</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -20372,24 +20372,24 @@
         <v>1</v>
       </c>
       <c r="M236" t="n">
-        <v>-58.490576</v>
+        <v>-58.417002</v>
       </c>
       <c r="N236" t="n">
-        <v>-34.561508</v>
+        <v>-34.618613</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q236" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>ALM-B</t>
         </is>
       </c>
       <c r="R236" t="inlineStr">
@@ -20401,7 +20401,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>00317296</t>
+          <t>00322642</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -20411,7 +20411,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>AGRELO 3620</t>
+          <t>ESTADO DE PALESTINA 727</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -20454,10 +20454,10 @@
         <v>1</v>
       </c>
       <c r="M237" t="n">
-        <v>-58.417002</v>
+        <v>-58.425539</v>
       </c>
       <c r="N237" t="n">
-        <v>-34.618613</v>
+        <v>-34.602286</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -20471,7 +20471,7 @@
       </c>
       <c r="Q237" t="inlineStr">
         <is>
-          <t>ALM-B</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R237" t="inlineStr">
@@ -20483,7 +20483,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>00322642</t>
+          <t>8263</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -20493,7 +20493,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>ESTADO DE PALESTINA 727</t>
+          <t>MEXICO 3306</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -20536,10 +20536,10 @@
         <v>1</v>
       </c>
       <c r="M238" t="n">
-        <v>-58.425539</v>
+        <v>-58.412865</v>
       </c>
       <c r="N238" t="n">
-        <v>-34.602286</v>
+        <v>-34.619484</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -20553,7 +20553,7 @@
       </c>
       <c r="Q238" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>CEN-J</t>
         </is>
       </c>
       <c r="R238" t="inlineStr">
@@ -20565,7 +20565,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>8263</t>
+          <t>8265</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -20575,12 +20575,12 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>MEXICO 3306</t>
+          <t>HUMBERTO 1 1999</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -20618,14 +20618,14 @@
         <v>1</v>
       </c>
       <c r="M239" t="n">
-        <v>-58.412865</v>
+        <v>-58.394304</v>
       </c>
       <c r="N239" t="n">
-        <v>-34.619484</v>
+        <v>-34.621645</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P239" t="inlineStr">
@@ -20635,7 +20635,7 @@
       </c>
       <c r="Q239" t="inlineStr">
         <is>
-          <t>CEN-J</t>
+          <t>CEN-B</t>
         </is>
       </c>
       <c r="R239" t="inlineStr">
@@ -20647,7 +20647,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>8265</t>
+          <t>08672</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -20657,12 +20657,12 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>HUMBERTO 1 1999</t>
+          <t>HERRERA 540</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -20688,7 +20688,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -20700,10 +20700,10 @@
         <v>1</v>
       </c>
       <c r="M240" t="n">
-        <v>-58.394304</v>
+        <v>-58.378264</v>
       </c>
       <c r="N240" t="n">
-        <v>-34.621645</v>
+        <v>-34.636021</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -20717,7 +20717,7 @@
       </c>
       <c r="Q240" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>CON-H</t>
         </is>
       </c>
       <c r="R240" t="inlineStr">
@@ -20729,22 +20729,22 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>08672</t>
+          <t>8647</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>3/23/2026</t>
+          <t>3/24/2026</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>HERRERA 540</t>
+          <t xml:space="preserve">MELIAN AV 4827 </t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -20760,7 +20760,7 @@
       <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -20782,24 +20782,24 @@
         <v>1</v>
       </c>
       <c r="M241" t="n">
-        <v>-58.378264</v>
+        <v>-58.487048</v>
       </c>
       <c r="N241" t="n">
-        <v>-34.636021</v>
+        <v>-34.545509</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>CON-H</t>
+          <t>COG-Q</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
@@ -20811,22 +20811,22 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>8647</t>
+          <t>8674</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>3/24/2026</t>
+          <t>3/23/2026</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t xml:space="preserve">MELIAN AV 4827 </t>
+          <t>BRASIL 2509</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -20842,7 +20842,7 @@
       <c r="G242" t="inlineStr"/>
       <c r="H242" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -20864,109 +20864,27 @@
         <v>1</v>
       </c>
       <c r="M242" t="n">
-        <v>-58.487048</v>
+        <v>-58.399415</v>
       </c>
       <c r="N242" t="n">
-        <v>-34.545509</v>
+        <v>-34.631112</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>COG-Q</t>
+          <t>PPT-F</t>
         </is>
       </c>
       <c r="R242" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>8674</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>3/23/2026</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>BRASIL 2509</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F243" t="inlineStr">
-        <is>
-          <t>Sin Asignar</t>
-        </is>
-      </c>
-      <c r="G243" t="inlineStr"/>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I243" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K243" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L243" t="n">
-        <v>1</v>
-      </c>
-      <c r="M243" t="n">
-        <v>-58.399415</v>
-      </c>
-      <c r="N243" t="n">
-        <v>-34.631112</v>
-      </c>
-      <c r="O243" t="inlineStr">
-        <is>
-          <t>San Telmo</t>
-        </is>
-      </c>
-      <c r="P243" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q243" t="inlineStr">
-        <is>
-          <t>PPT-F</t>
-        </is>
-      </c>
-      <c r="R243" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-28 12:28:54)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R242"/>
+  <dimension ref="A1:R245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20890,6 +20890,252 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11070617 </t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>3/28/2026</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>FONROUGE 1697</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L243" t="n">
+        <v>1</v>
+      </c>
+      <c r="M243" t="n">
+        <v>-58.496881</v>
+      </c>
+      <c r="N243" t="n">
+        <v>-34.653948</v>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>PAV-H</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>8703</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>3/28/2026</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>RIVADAVIA AV 1985</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>APLOMAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L244" t="n">
+        <v>1</v>
+      </c>
+      <c r="M244" t="n">
+        <v>-58.394609</v>
+      </c>
+      <c r="N244" t="n">
+        <v>-34.609304</v>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>CLI-B</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>8702</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>3/28/2026</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>JUNCAL 2249</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L245" t="n">
+        <v>1</v>
+      </c>
+      <c r="M245" t="n">
+        <v>-58.399319</v>
+      </c>
+      <c r="N245" t="n">
+        <v>-34.592221</v>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>RET-E</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.1RET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-16 09:13:21)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R143"/>
+  <dimension ref="A1:R147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12680,6 +12680,334 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>S00356265</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>RIVADAVIA MARTIN, COMODORO 2087</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>1</v>
+      </c>
+      <c r="M144" t="n">
+        <v>-58.465653</v>
+      </c>
+      <c r="N144" t="n">
+        <v>-34.546494</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>BLO-R</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>S00387253</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>DIAZ, CESAR, GRAL. 4881</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L145" t="n">
+        <v>1</v>
+      </c>
+      <c r="M145" t="n">
+        <v>-58.49779</v>
+      </c>
+      <c r="N145" t="n">
+        <v>-34.627626</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>DEV-I</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>S00396906</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>MARSELLA 2546</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>1</v>
+      </c>
+      <c r="M146" t="n">
+        <v>-58.477848</v>
+      </c>
+      <c r="N146" t="n">
+        <v>-34.582559</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>ATH-S</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>S00400580</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>4/14/2026</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>BORDABEHERE, ENZO 2802</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>1</v>
+      </c>
+      <c r="M147" t="n">
+        <v>-58.480405</v>
+      </c>
+      <c r="N147" t="n">
+        <v>-34.600087</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>PUE-A</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-20 12:36:56)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R147"/>
+  <dimension ref="A1:R184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13008,6 +13008,2964 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>EXPOSITO</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>JOSE CUBAS 2708</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Corer a línea de medianera por construcción de garage en vecino.</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L148" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" t="n">
+        <v>-58.497958</v>
+      </c>
+      <c r="N148" t="n">
+        <v>-34.587254</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>PUE-K</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>HALVAREZ</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ASUNCION 3719</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Poste quebrado en la base. Sostenido por tendido de red telecom. Con clientes activos</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="n">
+        <v>-58.5078</v>
+      </c>
+      <c r="N149" t="n">
+        <v>-34.598769</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>PUE-P</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>MI00001</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>LUGONES 2362</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
+        <v>-58.479067</v>
+      </c>
+      <c r="N150" t="n">
+        <v>-34.571679</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>ATH-E</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>GG0001</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>AV CABILDO 918</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Cambiar columna 114 golpeada provocando dobladora a 1mts del piso.</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="n">
+        <v>-58.445962</v>
+      </c>
+      <c r="N151" t="n">
+        <v>-34.569552</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>COG-C</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr"/>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" t="n">
+        <v>-58.444908</v>
+      </c>
+      <c r="N152" t="n">
+        <v>-34.607205</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr"/>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-58.419576</v>
+      </c>
+      <c r="N153" t="n">
+        <v>-34.621289</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr"/>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="n">
+        <v>-58.430568</v>
+      </c>
+      <c r="N154" t="n">
+        <v>-34.599485</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>CLI-N</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr"/>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" t="n">
+        <v>-58.437499</v>
+      </c>
+      <c r="N155" t="n">
+        <v>-34.578324</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr"/>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>1</v>
+      </c>
+      <c r="M156" t="n">
+        <v>-58.435547</v>
+      </c>
+      <c r="N156" t="n">
+        <v>-34.576622</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr"/>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>AREVALO 2006</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>1</v>
+      </c>
+      <c r="M157" t="n">
+        <v>-58.373629</v>
+      </c>
+      <c r="N157" t="n">
+        <v>-34.64417</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>CON-A</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>ARATO-25058.AF.1CON</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr"/>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L158" t="n">
+        <v>1</v>
+      </c>
+      <c r="M158" t="n">
+        <v>-58.444908</v>
+      </c>
+      <c r="N158" t="n">
+        <v>-34.607205</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr"/>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L159" t="n">
+        <v>1</v>
+      </c>
+      <c r="M159" t="n">
+        <v>-58.419576</v>
+      </c>
+      <c r="N159" t="n">
+        <v>-34.621289</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>1</v>
+      </c>
+      <c r="M160" t="n">
+        <v>-58.430568</v>
+      </c>
+      <c r="N160" t="n">
+        <v>-34.599485</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>CLI-N</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr"/>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>1</v>
+      </c>
+      <c r="M161" t="n">
+        <v>-58.437499</v>
+      </c>
+      <c r="N161" t="n">
+        <v>-34.578324</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr"/>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L162" t="n">
+        <v>1</v>
+      </c>
+      <c r="M162" t="n">
+        <v>-58.435547</v>
+      </c>
+      <c r="N162" t="n">
+        <v>-34.576622</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr"/>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>AREVALO 2260</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>1</v>
+      </c>
+      <c r="M163" t="n">
+        <v>-58.373629</v>
+      </c>
+      <c r="N163" t="n">
+        <v>-34.64417</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>CON-A</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>ARATO-25058.AF.1CON</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr"/>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>1</v>
+      </c>
+      <c r="M164" t="n">
+        <v>-58.444908</v>
+      </c>
+      <c r="N164" t="n">
+        <v>-34.607205</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>ALM-O</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr"/>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>1</v>
+      </c>
+      <c r="M165" t="n">
+        <v>-58.419576</v>
+      </c>
+      <c r="N165" t="n">
+        <v>-34.621289</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr"/>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" t="n">
+        <v>-58.430568</v>
+      </c>
+      <c r="N166" t="n">
+        <v>-34.599485</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>CLI-N</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr"/>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L167" t="n">
+        <v>1</v>
+      </c>
+      <c r="M167" t="n">
+        <v>-58.437499</v>
+      </c>
+      <c r="N167" t="n">
+        <v>-34.578324</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr"/>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>1</v>
+      </c>
+      <c r="M168" t="n">
+        <v>-58.435547</v>
+      </c>
+      <c r="N168" t="n">
+        <v>-34.576622</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>ATH-B</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr"/>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>MONTES DE OCA, MANUEL AV. 1441</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="n">
+        <v>-58.373629</v>
+      </c>
+      <c r="N169" t="n">
+        <v>-34.64417</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>CON-A</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>ARATO-25058.AF.1CON</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>AL00001</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>ALVAREZ THOMAS AV. 1270</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="n">
+        <v>-58.459453</v>
+      </c>
+      <c r="N170" t="n">
+        <v>-34.57843</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>ATH-O</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>GG00003</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>PEDRAZA, MANUELA 2649</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>1</v>
+      </c>
+      <c r="M171" t="n">
+        <v>-58.468626</v>
+      </c>
+      <c r="N171" t="n">
+        <v>-34.552938</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>COG-L</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>PJ00009</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>THAMES 1516</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>1</v>
+      </c>
+      <c r="M172" t="n">
+        <v>-58.431966</v>
+      </c>
+      <c r="N172" t="n">
+        <v>-34.588553</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>VCR-F</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>HT00001</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>CURUPAYTI 2997</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>1</v>
+      </c>
+      <c r="M173" t="n">
+        <v>-58.508912</v>
+      </c>
+      <c r="N173" t="n">
+        <v>-34.580858</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>PUE-J</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>LR00001</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr"/>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>BILLINGHURST 1796</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L174" t="n">
+        <v>1</v>
+      </c>
+      <c r="M174" t="n">
+        <v>-58.409695</v>
+      </c>
+      <c r="N174" t="n">
+        <v>-34.589662</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>AGU-D</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>PJ00040</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>HONDURAS 4822</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L175" t="n">
+        <v>1</v>
+      </c>
+      <c r="M175" t="n">
+        <v>-58.428528</v>
+      </c>
+      <c r="N175" t="n">
+        <v>-34.589872</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>VCR-F</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>AF00001</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>SALGUERO, JERONIMO 1995</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L176" t="n">
+        <v>1</v>
+      </c>
+      <c r="M176" t="n">
+        <v>-58.413378</v>
+      </c>
+      <c r="N176" t="n">
+        <v>-34.587254</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>VCR-G</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>AL00050</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>CULLEN 5771</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>1</v>
+      </c>
+      <c r="M177" t="n">
+        <v>-58.49549</v>
+      </c>
+      <c r="N177" t="n">
+        <v>-34.577008</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>PUE-I</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>RB00001</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>BELGRANO AV. 3715</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M178" t="n">
+        <v>-58.418851</v>
+      </c>
+      <c r="N178" t="n">
+        <v>-34.615716</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>ALM-C</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>AM00001</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>ARAUJO 2416</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>1</v>
+      </c>
+      <c r="M179" t="n">
+        <v>-58.481107</v>
+      </c>
+      <c r="N179" t="n">
+        <v>-34.659759</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>PAV-O</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>GG00035</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>FIGUEROA, D. APOLINARIO, CORONEL 1793</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>APLOMAR</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>1</v>
+      </c>
+      <c r="M180" t="n">
+        <v>-58.461005</v>
+      </c>
+      <c r="N180" t="n">
+        <v>-34.613152</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>NRA-J</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>AM00039</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>CASTRO BARROS 852</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>1</v>
+      </c>
+      <c r="M181" t="n">
+        <v>-58.419281</v>
+      </c>
+      <c r="N181" t="n">
+        <v>-34.62215</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>LR00044</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>CHARCAS 3250</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>1</v>
+      </c>
+      <c r="M182" t="n">
+        <v>-58.41175</v>
+      </c>
+      <c r="N182" t="n">
+        <v>-34.592173</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>AGU-C</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>RB12120</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>CERRI, DANIEL, GRAL. 1214</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>1</v>
+      </c>
+      <c r="M183" t="n">
+        <v>-58.366979</v>
+      </c>
+      <c r="N183" t="n">
+        <v>-34.646341</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>CON-E</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>AL25250</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>4/20/2026</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>ARENAL, CONCEPCION 3526</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L184" t="n">
+        <v>1</v>
+      </c>
+      <c r="M184" t="n">
+        <v>-58.446573</v>
+      </c>
+      <c r="N184" t="n">
+        <v>-34.5842</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>ATH-L</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-22 11:36:13)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Sin_Asignar.xlsx
+++ b/mapa_interactivo_Sin_Asignar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R210"/>
+  <dimension ref="A1:R224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13139,7 +13139,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M149" t="n">
         <v>-58.479067</v>
@@ -18073,6 +18073,1154 @@
         </is>
       </c>
       <c r="R210" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>S00299569</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>YRIGOYEN, HIPOLITO AV. 4156</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L211" t="n">
+        <v>1</v>
+      </c>
+      <c r="M211" t="n">
+        <v>-58.425213</v>
+      </c>
+      <c r="N211" t="n">
+        <v>-34.614924</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>ALM-D</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>S004318770</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>SARMIENTO 4290</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr"/>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L212" t="n">
+        <v>1</v>
+      </c>
+      <c r="M212" t="n">
+        <v>-58.425764</v>
+      </c>
+      <c r="N212" t="n">
+        <v>-34.604359</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>ALM-L</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>S00431893</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>MUÑIZ 1151</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L213" t="n">
+        <v>1</v>
+      </c>
+      <c r="M213" t="n">
+        <v>-58.425442</v>
+      </c>
+      <c r="N213" t="n">
+        <v>-34.627634</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>PPT-P</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>S00434849</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>YRIGOYEN, HIPOLITO AV. 3484</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L214" t="n">
+        <v>1</v>
+      </c>
+      <c r="M214" t="n">
+        <v>-58.416028</v>
+      </c>
+      <c r="N214" t="n">
+        <v>-34.613538</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>CEN-J</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9009 </t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>SANCHEZ DE LORIA 1913</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>1</v>
+      </c>
+      <c r="M215" t="n">
+        <v>-58.411474</v>
+      </c>
+      <c r="N215" t="n">
+        <v>-34.633143</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>PPT-Q</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9011 </t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>SANCHEZ DE LORIA 1583</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>1</v>
+      </c>
+      <c r="M216" t="n">
+        <v>-58.411926</v>
+      </c>
+      <c r="N216" t="n">
+        <v>-34.628861</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>PPT-E</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9012 </t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LINIERS VIRREY 2315 </t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>1</v>
+      </c>
+      <c r="M217" t="n">
+        <v>-58.41191</v>
+      </c>
+      <c r="N217" t="n">
+        <v>-34.637333</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>PPT-Q</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9014 </t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>LINIERS VIRREY 896</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>1</v>
+      </c>
+      <c r="M218" t="n">
+        <v>-58.413645</v>
+      </c>
+      <c r="N218" t="n">
+        <v>-34.621935</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>CEN-P</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9016 </t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>HUMBERTO 1° 3368</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L219" t="n">
+        <v>1</v>
+      </c>
+      <c r="M219" t="n">
+        <v>-58.413189</v>
+      </c>
+      <c r="N219" t="n">
+        <v>-34.624187</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>CEN-P</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9017 </t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>MUÑIZ 1237</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L220" t="n">
+        <v>1</v>
+      </c>
+      <c r="M220" t="n">
+        <v>-58.425206</v>
+      </c>
+      <c r="N220" t="n">
+        <v>-34.628705</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>PPT-P</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9020 </t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>TARIJA 3497</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L221" t="n">
+        <v>1</v>
+      </c>
+      <c r="M221" t="n">
+        <v>-58.414424</v>
+      </c>
+      <c r="N221" t="n">
+        <v>-34.628778</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>PPT-E</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>S00378456</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>FRAY CAYETANO RODRIGUEZ 99</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L222" t="n">
+        <v>1</v>
+      </c>
+      <c r="M222" t="n">
+        <v>-58.463098</v>
+      </c>
+      <c r="N222" t="n">
+        <v>-34.627733</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>PCH-H</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>S00334047</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>SAN JOSE DE CALASANZ 755</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L223" t="n">
+        <v>1</v>
+      </c>
+      <c r="M223" t="n">
+        <v>-58.437351</v>
+      </c>
+      <c r="N223" t="n">
+        <v>-34.627956</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>PCH-C</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>S0000223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>4/21/2026</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>ARENALES 3660</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L224" t="n">
+        <v>1</v>
+      </c>
+      <c r="M224" t="n">
+        <v>-58.413732</v>
+      </c>
+      <c r="N224" t="n">
+        <v>-34.585415</v>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>AGU-L</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>